<commit_message>
cambios en arduino MEGA de depuracion de sensores
</commit_message>
<xml_diff>
--- a/conexiones entrada y salida.xlsx
+++ b/conexiones entrada y salida.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://365udit-my.sharepoint.com/personal/javier_fernandezdegorostiza_udit_es/Documents/dartecne/isla de los sonidos/isla de los sonidos/sonido/doc/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://365udit-my.sharepoint.com/personal/javier_fernandezdegorostiza_udit_es/Documents/src/LISA/src/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="75" documentId="8_{75FAB1E9-A2F1-481D-93AF-E273F04992DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB3B3403-D2C9-43C9-9548-69A48037B18D}"/>
+  <xr:revisionPtr revIDLastSave="76" documentId="8_{75FAB1E9-A2F1-481D-93AF-E273F04992DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06DF5430-631E-49A0-9C27-7E0C92F96FF6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C02A2D68-7A3C-44F3-BE09-91F50885F2CC}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="194">
   <si>
     <t>Arduino MEGA</t>
   </si>
@@ -961,9 +961,6 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1011,6 +1008,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="18">
@@ -1502,7 +1502,7 @@
       <c r="A4" s="3"/>
       <c r="B4"/>
       <c r="C4" s="1"/>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="14" t="s">
         <v>110</v>
       </c>
       <c r="E4" s="3"/>
@@ -2736,7 +2736,7 @@
       <c r="C13" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="15" t="s">
         <v>114</v>
       </c>
       <c r="F13" s="8" t="s">
@@ -2763,7 +2763,7 @@
       <c r="C14" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="D14" s="16" t="s">
+      <c r="D14" s="15" t="s">
         <v>118</v>
       </c>
       <c r="F14" s="8" t="s">
@@ -2781,15 +2781,15 @@
       <c r="L14" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="M14" s="14" t="s">
-        <v>77</v>
+      <c r="M14" s="30">
+        <v>46274</v>
       </c>
     </row>
     <row r="15" spans="1:1025 16383:16384">
       <c r="C15" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="D15" s="16" t="s">
+      <c r="D15" s="15" t="s">
         <v>122</v>
       </c>
       <c r="F15" s="8" t="s">
@@ -2815,7 +2815,7 @@
       <c r="C16" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="D16" s="16" t="s">
+      <c r="D16" s="15" t="s">
         <v>126</v>
       </c>
       <c r="F16" s="8" t="s">
@@ -2841,7 +2841,7 @@
       <c r="C17" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="D17" s="16" t="s">
+      <c r="D17" s="15" t="s">
         <v>129</v>
       </c>
       <c r="F17" s="8" t="s">
@@ -2867,7 +2867,7 @@
       <c r="C18" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="D18" s="16" t="s">
+      <c r="D18" s="15" t="s">
         <v>132</v>
       </c>
       <c r="F18" s="8" t="s">
@@ -2893,7 +2893,7 @@
       <c r="C19" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="D19" s="16" t="s">
+      <c r="D19" s="15" t="s">
         <v>135</v>
       </c>
       <c r="F19" s="3"/>
@@ -2917,7 +2917,7 @@
       <c r="C20" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="D20" s="16" t="s">
+      <c r="D20" s="15" t="s">
         <v>138</v>
       </c>
       <c r="F20" s="8" t="s">
@@ -3012,501 +3012,501 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="10.69921875" customWidth="1"/>
-    <col min="2" max="2" width="24.296875" style="17" customWidth="1"/>
-    <col min="3" max="3" width="14" style="17" customWidth="1"/>
-    <col min="4" max="4" width="7.19921875" style="18" customWidth="1"/>
-    <col min="5" max="5" width="5.296875" style="18" customWidth="1"/>
-    <col min="6" max="6" width="16.8984375" style="19" customWidth="1"/>
-    <col min="7" max="7" width="17.296875" style="17" customWidth="1"/>
+    <col min="2" max="2" width="24.296875" style="16" customWidth="1"/>
+    <col min="3" max="3" width="14" style="16" customWidth="1"/>
+    <col min="4" max="4" width="7.19921875" style="17" customWidth="1"/>
+    <col min="5" max="5" width="5.296875" style="17" customWidth="1"/>
+    <col min="6" max="6" width="16.8984375" style="18" customWidth="1"/>
+    <col min="7" max="7" width="17.296875" style="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:7">
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="28" t="s">
         <v>139</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="22" t="s">
+      <c r="C3" s="19"/>
+      <c r="D3" s="21" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="4" spans="2:7">
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="21" t="s">
         <v>174</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="21" t="s">
         <v>175</v>
       </c>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="22" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="5" spans="2:7">
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="C5" s="23" t="s">
         <v>144</v>
       </c>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="26"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="25"/>
     </row>
     <row r="6" spans="2:7">
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="23" t="s">
         <v>146</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="23" t="s">
         <v>147</v>
       </c>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="26" t="s">
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="25" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="7" spans="2:7">
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="23" t="s">
         <v>188</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="C7" s="23" t="s">
         <v>148</v>
       </c>
-      <c r="D7" s="25" t="s">
+      <c r="D7" s="24" t="s">
         <v>178</v>
       </c>
-      <c r="E7" s="25">
+      <c r="E7" s="24">
         <v>1</v>
       </c>
-      <c r="F7" s="26">
+      <c r="F7" s="25">
         <v>12.13</v>
       </c>
     </row>
     <row r="10" spans="2:7">
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="28" t="s">
         <v>150</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="21" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="11" spans="2:7">
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="C11" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="D11" s="22" t="s">
+      <c r="D11" s="21" t="s">
         <v>174</v>
       </c>
-      <c r="E11" s="22" t="s">
+      <c r="E11" s="21" t="s">
         <v>175</v>
       </c>
-      <c r="F11" s="23" t="s">
+      <c r="F11" s="22" t="s">
         <v>176</v>
       </c>
-      <c r="G11" s="22" t="s">
+      <c r="G11" s="21" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="12" spans="2:7">
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="23" t="s">
         <v>152</v>
       </c>
-      <c r="C12" s="24" t="s">
+      <c r="C12" s="23" t="s">
         <v>153</v>
       </c>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="23"/>
     </row>
     <row r="13" spans="2:7" ht="27.6">
-      <c r="B13" s="24" t="s">
+      <c r="B13" s="23" t="s">
         <v>155</v>
       </c>
-      <c r="C13" s="24" t="s">
+      <c r="C13" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="D13" s="25" t="s">
+      <c r="D13" s="24" t="s">
         <v>179</v>
       </c>
-      <c r="E13" s="25">
+      <c r="E13" s="24">
         <v>1</v>
       </c>
-      <c r="F13" s="26" t="s">
+      <c r="F13" s="25" t="s">
         <v>180</v>
       </c>
-      <c r="G13" s="24"/>
+      <c r="G13" s="23"/>
     </row>
     <row r="14" spans="2:7">
-      <c r="B14" s="24" t="s">
+      <c r="B14" s="23" t="s">
         <v>157</v>
       </c>
-      <c r="C14" s="24" t="s">
+      <c r="C14" s="23" t="s">
         <v>158</v>
       </c>
-      <c r="D14" s="25" t="s">
+      <c r="D14" s="24" t="s">
         <v>181</v>
       </c>
-      <c r="E14" s="25" t="s">
+      <c r="E14" s="24" t="s">
         <v>181</v>
       </c>
-      <c r="F14" s="26" t="s">
+      <c r="F14" s="25" t="s">
         <v>181</v>
       </c>
-      <c r="G14" s="24"/>
+      <c r="G14" s="23"/>
     </row>
     <row r="15" spans="2:7">
-      <c r="B15" s="24" t="s">
+      <c r="B15" s="23" t="s">
         <v>189</v>
       </c>
-      <c r="C15" s="27" t="s">
+      <c r="C15" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="D15" s="25" t="s">
+      <c r="D15" s="24" t="s">
         <v>178</v>
       </c>
-      <c r="E15" s="25">
+      <c r="E15" s="24">
         <v>1</v>
       </c>
-      <c r="F15" s="26">
+      <c r="F15" s="25">
         <v>14</v>
       </c>
-      <c r="G15" s="24"/>
+      <c r="G15" s="23"/>
     </row>
     <row r="16" spans="2:7">
-      <c r="B16" s="24"/>
-      <c r="C16" s="28" t="s">
+      <c r="B16" s="23"/>
+      <c r="C16" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="23"/>
     </row>
     <row r="17" spans="2:7">
-      <c r="B17" s="24"/>
-      <c r="C17" s="28" t="s">
+      <c r="B17" s="23"/>
+      <c r="C17" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="23"/>
     </row>
     <row r="18" spans="2:7">
-      <c r="B18" s="24" t="s">
+      <c r="B18" s="23" t="s">
         <v>190</v>
       </c>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="D18" s="25" t="s">
+      <c r="D18" s="24" t="s">
         <v>178</v>
       </c>
-      <c r="E18" s="25">
+      <c r="E18" s="24">
         <v>1</v>
       </c>
-      <c r="F18" s="26">
+      <c r="F18" s="25">
         <v>15</v>
       </c>
-      <c r="G18" s="24"/>
+      <c r="G18" s="23"/>
     </row>
     <row r="19" spans="2:7">
-      <c r="B19" s="24"/>
-      <c r="C19" s="28" t="s">
+      <c r="B19" s="23"/>
+      <c r="C19" s="27" t="s">
         <v>53</v>
       </c>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="25"/>
+      <c r="G19" s="23"/>
     </row>
     <row r="20" spans="2:7">
-      <c r="B20" s="24"/>
-      <c r="C20" s="30" t="s">
+      <c r="B20" s="23"/>
+      <c r="C20" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="25"/>
+      <c r="G20" s="23"/>
     </row>
     <row r="22" spans="2:7">
-      <c r="B22" s="29" t="s">
+      <c r="B22" s="28" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="23" spans="2:7">
-      <c r="B23" s="21" t="s">
+      <c r="B23" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="C23" s="21" t="s">
+      <c r="C23" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="26"/>
-      <c r="G23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="25"/>
+      <c r="G23" s="23"/>
     </row>
     <row r="24" spans="2:7">
-      <c r="B24" s="24" t="s">
+      <c r="B24" s="23" t="s">
         <v>164</v>
       </c>
-      <c r="C24" s="24" t="s">
+      <c r="C24" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="26"/>
-      <c r="G24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="25"/>
+      <c r="G24" s="23"/>
     </row>
     <row r="25" spans="2:7">
-      <c r="B25" s="24" t="s">
+      <c r="B25" s="23" t="s">
         <v>165</v>
       </c>
-      <c r="C25" s="24" t="s">
+      <c r="C25" s="23" t="s">
         <v>166</v>
       </c>
-      <c r="D25" s="25"/>
-      <c r="E25" s="25"/>
-      <c r="F25" s="26"/>
-      <c r="G25" s="24"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="25"/>
+      <c r="G25" s="23"/>
     </row>
     <row r="26" spans="2:7">
-      <c r="B26" s="24" t="s">
+      <c r="B26" s="23" t="s">
         <v>167</v>
       </c>
-      <c r="C26" s="24" t="s">
+      <c r="C26" s="23" t="s">
         <v>168</v>
       </c>
-      <c r="D26" s="25"/>
-      <c r="E26" s="25"/>
-      <c r="F26" s="26"/>
-      <c r="G26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="25"/>
+      <c r="G26" s="23"/>
     </row>
     <row r="27" spans="2:7">
-      <c r="B27" s="24" t="s">
+      <c r="B27" s="23" t="s">
         <v>169</v>
       </c>
-      <c r="C27" s="24" t="s">
+      <c r="C27" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="D27" s="25"/>
-      <c r="E27" s="25"/>
-      <c r="F27" s="26"/>
-      <c r="G27" s="24"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="25"/>
+      <c r="G27" s="23"/>
     </row>
     <row r="28" spans="2:7">
-      <c r="B28" s="24" t="s">
+      <c r="B28" s="23" t="s">
         <v>170</v>
       </c>
-      <c r="C28" s="24" t="s">
+      <c r="C28" s="23" t="s">
         <v>124</v>
       </c>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="26"/>
-      <c r="G28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="25"/>
+      <c r="G28" s="23"/>
     </row>
     <row r="29" spans="2:7">
-      <c r="B29" s="24" t="s">
+      <c r="B29" s="23" t="s">
         <v>171</v>
       </c>
-      <c r="C29" s="24" t="s">
+      <c r="C29" s="23" t="s">
         <v>172</v>
       </c>
-      <c r="D29" s="25"/>
-      <c r="E29" s="25"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="24"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="25"/>
+      <c r="G29" s="23"/>
     </row>
     <row r="31" spans="2:7">
-      <c r="B31" s="29" t="s">
+      <c r="B31" s="28" t="s">
         <v>140</v>
       </c>
-      <c r="D31" s="22" t="s">
+      <c r="D31" s="21" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="32" spans="2:7">
-      <c r="B32" s="21" t="s">
+      <c r="B32" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="C32" s="21" t="s">
+      <c r="C32" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="D32" s="22" t="s">
+      <c r="D32" s="21" t="s">
         <v>174</v>
       </c>
-      <c r="E32" s="22" t="s">
+      <c r="E32" s="21" t="s">
         <v>175</v>
       </c>
-      <c r="F32" s="23" t="s">
+      <c r="F32" s="22" t="s">
         <v>176</v>
       </c>
-      <c r="G32" s="22" t="s">
+      <c r="G32" s="21" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="33" spans="2:7">
-      <c r="B33" s="24" t="s">
+      <c r="B33" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="C33" s="24" t="s">
+      <c r="C33" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="D33" s="25"/>
-      <c r="E33" s="25"/>
-      <c r="F33" s="26"/>
-      <c r="G33" s="24"/>
+      <c r="D33" s="24"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="25"/>
+      <c r="G33" s="23"/>
     </row>
     <row r="35" spans="2:7">
-      <c r="B35" s="29" t="s">
+      <c r="B35" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="D35" s="22" t="s">
+      <c r="D35" s="21" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="36" spans="2:7">
-      <c r="B36" s="21" t="s">
+      <c r="B36" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="C36" s="21" t="s">
+      <c r="C36" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="D36" s="22" t="s">
+      <c r="D36" s="21" t="s">
         <v>174</v>
       </c>
-      <c r="E36" s="22" t="s">
+      <c r="E36" s="21" t="s">
         <v>175</v>
       </c>
-      <c r="F36" s="23" t="s">
+      <c r="F36" s="22" t="s">
         <v>176</v>
       </c>
-      <c r="G36" s="22" t="s">
+      <c r="G36" s="21" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="37" spans="2:7">
-      <c r="B37" s="24" t="s">
+      <c r="B37" s="23" t="s">
         <v>151</v>
       </c>
-      <c r="C37" s="24" t="s">
+      <c r="C37" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="D37" s="25" t="s">
+      <c r="D37" s="24" t="s">
         <v>179</v>
       </c>
-      <c r="E37" s="25">
+      <c r="E37" s="24">
         <v>1</v>
       </c>
-      <c r="F37" s="26" t="s">
+      <c r="F37" s="25" t="s">
         <v>183</v>
       </c>
-      <c r="G37" s="24" t="s">
+      <c r="G37" s="23" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="38" spans="2:7">
-      <c r="B38" s="24"/>
-      <c r="C38" s="24"/>
-      <c r="D38" s="25" t="s">
+      <c r="B38" s="23"/>
+      <c r="C38" s="23"/>
+      <c r="D38" s="24" t="s">
         <v>179</v>
       </c>
-      <c r="E38" s="25">
+      <c r="E38" s="24">
         <v>1</v>
       </c>
-      <c r="F38" s="26" t="s">
+      <c r="F38" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="G38" s="24" t="s">
+      <c r="G38" s="23" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="39" spans="2:7">
-      <c r="B39" s="24"/>
-      <c r="C39" s="24"/>
-      <c r="D39" s="25" t="s">
+      <c r="B39" s="23"/>
+      <c r="C39" s="23"/>
+      <c r="D39" s="24" t="s">
         <v>179</v>
       </c>
-      <c r="E39" s="25">
+      <c r="E39" s="24">
         <v>1</v>
       </c>
-      <c r="F39" s="26" t="s">
+      <c r="F39" s="25" t="s">
         <v>186</v>
       </c>
-      <c r="G39" s="24" t="s">
+      <c r="G39" s="23" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="41" spans="2:7">
-      <c r="B41" s="29" t="s">
+      <c r="B41" s="28" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="42" spans="2:7">
-      <c r="B42" s="21" t="s">
+      <c r="B42" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="C42" s="21" t="s">
+      <c r="C42" s="20" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="43" spans="2:7">
-      <c r="B43" s="24" t="s">
+      <c r="B43" s="23" t="s">
         <v>159</v>
       </c>
-      <c r="C43" s="24" t="s">
+      <c r="C43" s="23" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="45" spans="2:7">
-      <c r="B45" s="29" t="s">
+      <c r="B45" s="28" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="46" spans="2:7">
-      <c r="B46" s="21" t="s">
+      <c r="B46" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="C46" s="21" t="s">
+      <c r="C46" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="D46" s="25"/>
-      <c r="E46" s="25"/>
-      <c r="F46" s="26"/>
-      <c r="G46" s="24"/>
+      <c r="D46" s="24"/>
+      <c r="E46" s="24"/>
+      <c r="F46" s="25"/>
+      <c r="G46" s="23"/>
     </row>
     <row r="47" spans="2:7">
-      <c r="B47" s="24" t="s">
+      <c r="B47" s="23" t="s">
         <v>163</v>
       </c>
-      <c r="C47" s="24" t="s">
+      <c r="C47" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="D47" s="25"/>
-      <c r="E47" s="25"/>
-      <c r="F47" s="26"/>
-      <c r="G47" s="24"/>
+      <c r="D47" s="24"/>
+      <c r="E47" s="24"/>
+      <c r="F47" s="25"/>
+      <c r="G47" s="23"/>
     </row>
     <row r="48" spans="2:7">
-      <c r="B48" s="24"/>
-      <c r="C48" s="24" t="s">
+      <c r="B48" s="23"/>
+      <c r="C48" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="D48" s="25"/>
-      <c r="E48" s="25"/>
-      <c r="F48" s="26"/>
-      <c r="G48" s="24"/>
+      <c r="D48" s="24"/>
+      <c r="E48" s="24"/>
+      <c r="F48" s="25"/>
+      <c r="G48" s="23"/>
     </row>
   </sheetData>
   <pageMargins left="0" right="0" top="0.39370078740157505" bottom="0.39370078740157505" header="0" footer="0"/>

</xml_diff>

<commit_message>
arduino wemos stones and bambus
</commit_message>
<xml_diff>
--- a/conexiones entrada y salida.xlsx
+++ b/conexiones entrada y salida.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://365udit-my.sharepoint.com/personal/javier_fernandezdegorostiza_udit_es/Documents/src/LISA/src/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="76" documentId="8_{75FAB1E9-A2F1-481D-93AF-E273F04992DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06DF5430-631E-49A0-9C27-7E0C92F96FF6}"/>
+  <xr:revisionPtr revIDLastSave="158" documentId="8_{75FAB1E9-A2F1-481D-93AF-E273F04992DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7DE8781-AEB3-49C7-A596-30E5B1A9548F}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C02A2D68-7A3C-44F3-BE09-91F50885F2CC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C02A2D68-7A3C-44F3-BE09-91F50885F2CC}"/>
   </bookViews>
   <sheets>
     <sheet name="Arduino_MEGA_v2" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="195">
   <si>
     <t>Arduino MEGA</t>
   </si>
@@ -372,27 +372,15 @@
     <t>A0</t>
   </si>
   <si>
-    <t>pot_1</t>
-  </si>
-  <si>
     <t>A8</t>
   </si>
   <si>
-    <t>joy_x</t>
-  </si>
-  <si>
     <t>A1</t>
   </si>
   <si>
-    <t>pot_2</t>
-  </si>
-  <si>
     <t>A9</t>
   </si>
   <si>
-    <t>joy_y</t>
-  </si>
-  <si>
     <t>A2</t>
   </si>
   <si>
@@ -402,9 +390,6 @@
     <t>A10</t>
   </si>
   <si>
-    <t>puente_piezo[0]</t>
-  </si>
-  <si>
     <t>A3</t>
   </si>
   <si>
@@ -414,45 +399,30 @@
     <t>A11</t>
   </si>
   <si>
-    <t>puente_piezo[1]</t>
-  </si>
-  <si>
     <t>A4</t>
   </si>
   <si>
     <t>A12</t>
   </si>
   <si>
-    <t>puente_piezo[2]</t>
-  </si>
-  <si>
     <t>A5</t>
   </si>
   <si>
     <t>A13</t>
   </si>
   <si>
-    <t>puente_piezo[3]</t>
-  </si>
-  <si>
     <t>A6</t>
   </si>
   <si>
     <t>A14</t>
   </si>
   <si>
-    <t>puente_piezo[4]</t>
-  </si>
-  <si>
     <t>A7</t>
   </si>
   <si>
     <t>A15</t>
   </si>
   <si>
-    <t>puente_piezo[5]</t>
-  </si>
-  <si>
     <t>Ambiente Isla</t>
   </si>
   <si>
@@ -616,13 +586,46 @@
   </si>
   <si>
     <t>NC</t>
+  </si>
+  <si>
+    <t>MIC</t>
+  </si>
+  <si>
+    <t>MIDI NOTE</t>
+  </si>
+  <si>
+    <t>MIDI CC</t>
+  </si>
+  <si>
+    <t>[60, 61, 62, 63, 64, 65]</t>
+  </si>
+  <si>
+    <t>36,44,52</t>
+  </si>
+  <si>
+    <t>37,45,53</t>
+  </si>
+  <si>
+    <t>41,49,57</t>
+  </si>
+  <si>
+    <t>38...</t>
+  </si>
+  <si>
+    <t>39...</t>
+  </si>
+  <si>
+    <t>40...</t>
+  </si>
+  <si>
+    <t>--</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -721,8 +724,19 @@
       <color theme="1"/>
       <name val="Liberation Sans"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Liberation Sans"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -795,8 +809,44 @@
         <bgColor rgb="FFBEE3D3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -852,17 +902,6 @@
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -899,6 +938,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -920,7 +979,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -940,31 +999,16 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -979,22 +1023,22 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1003,13 +1047,73 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="16" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1048,49 +1152,6 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="304796" cy="304796"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="AutoShape 2" descr="Arduino Mega 2560 Rev3 Pinout">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D6695FD7-000F-9082-802E-894DF7CDEB84}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="15716250" y="2371725"/>
-          <a:ext cx="304796" cy="304796"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln cap="flat">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:endParaRPr lang="es-ES"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -1100,9 +1161,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>4139458</xdr:colOff>
+      <xdr:colOff>4135648</xdr:colOff>
       <xdr:row>28</xdr:row>
-      <xdr:rowOff>144780</xdr:rowOff>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1134,6 +1195,67 @@
         <a:xfrm>
           <a:off x="0" y="0"/>
           <a:ext cx="4992898" cy="5364480"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1037167</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>116416</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>1122892</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>27517</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6405910F-6092-4077-6AD2-DFDC816018AF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="12075584" y="4138083"/>
+          <a:ext cx="6552141" cy="2504017"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1472,7 +1594,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63F7371A-2114-47DC-A54A-388A73790A71}">
-  <dimension ref="A2:XFD27"/>
+  <dimension ref="A2:XFD44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="11.19921875" style="1" customWidth="1"/>
@@ -1482,13 +1604,19 @@
     <col min="5" max="5" width="7.09765625" style="1" customWidth="1"/>
     <col min="6" max="6" width="4.796875" style="1" customWidth="1"/>
     <col min="7" max="7" width="14.3984375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="5.296875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="5.8984375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.19921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.796875" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.296875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="3.3984375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="4.19921875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="12.19921875" style="1" customWidth="1"/>
-    <col min="14" max="1025" width="10.69921875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="4.19921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.19921875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="7.796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.69921875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="4.19921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="17.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="7.796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="1025" width="10.69921875" style="1" customWidth="1"/>
     <col min="1026" max="16382" width="11.19921875" customWidth="1"/>
     <col min="16383" max="16384" width="11.19921875" style="1" customWidth="1"/>
   </cols>
@@ -1502,7 +1630,7 @@
       <c r="A4" s="3"/>
       <c r="B4"/>
       <c r="C4" s="1"/>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="9" t="s">
         <v>110</v>
       </c>
       <c r="E4" s="3"/>
@@ -1510,22 +1638,32 @@
       <c r="G4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="4" t="s">
+      <c r="H4" s="30" t="s">
+        <v>185</v>
+      </c>
+      <c r="I4" s="30" t="s">
+        <v>186</v>
+      </c>
+      <c r="K4" s="3"/>
+      <c r="L4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="4" t="s">
+      <c r="M4" s="30" t="s">
+        <v>185</v>
+      </c>
+      <c r="N4" s="30" t="s">
+        <v>186</v>
+      </c>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
+      <c r="R4" s="30" t="s">
+        <v>185</v>
+      </c>
+      <c r="S4" s="30" t="s">
+        <v>186</v>
+      </c>
       <c r="T4" s="3"/>
       <c r="U4" s="3"/>
       <c r="V4" s="3"/>
@@ -2536,464 +2674,595 @@
       <c r="XFD4" s="3"/>
     </row>
     <row r="5" spans="1:1025 16383:16384" ht="14.4">
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>112</v>
-      </c>
+      <c r="D5" s="25"/>
       <c r="F5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="H5" s="31"/>
+      <c r="I5" s="31"/>
+      <c r="K5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="J5" s="10" t="s">
+      <c r="L5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="L5" s="8" t="s">
+      <c r="M5" s="31"/>
+      <c r="N5" s="31"/>
+      <c r="P5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="M5" s="10" t="s">
+      <c r="Q5" s="41" t="s">
         <v>11</v>
       </c>
+      <c r="R5" s="31" t="s">
+        <v>188</v>
+      </c>
+      <c r="S5" s="31"/>
     </row>
     <row r="6" spans="1:1025 16383:16384" ht="14.4">
-      <c r="C6" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>116</v>
-      </c>
+      <c r="C6" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="D6" s="25"/>
       <c r="F6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="H6" s="31"/>
+      <c r="I6" s="31"/>
+      <c r="K6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="10" t="s">
+      <c r="L6" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="L6" s="8" t="s">
+      <c r="M6" s="31"/>
+      <c r="N6" s="31"/>
+      <c r="P6" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="M6" s="10" t="s">
+      <c r="Q6" s="41" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="7" spans="1:1025 16383:16384" ht="14.4">
-      <c r="C7" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>120</v>
-      </c>
+      <c r="R6" s="31" t="s">
+        <v>189</v>
+      </c>
+      <c r="S6" s="31"/>
+    </row>
+    <row r="7" spans="1:1025 16383:16384">
+      <c r="C7" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D7" s="25"/>
       <c r="F7" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="H7" s="31"/>
+      <c r="I7" s="31"/>
+      <c r="K7" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="J7" s="10" t="s">
-        <v>193</v>
-      </c>
-      <c r="K7" s="12"/>
       <c r="L7" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="M7" s="31"/>
+      <c r="N7" s="31"/>
+      <c r="P7" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="M7" s="10" t="s">
+      <c r="Q7" s="41" t="s">
         <v>27</v>
       </c>
+      <c r="R7" s="31" t="s">
+        <v>191</v>
+      </c>
+      <c r="S7" s="31"/>
     </row>
     <row r="8" spans="1:1025 16383:16384">
-      <c r="C8" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>124</v>
-      </c>
+      <c r="C8" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="D8" s="25"/>
       <c r="F8" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="G8" s="13" t="s">
+      <c r="G8" s="44" t="s">
         <v>29</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="H8" s="31"/>
+      <c r="I8" s="31"/>
+      <c r="K8" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="J8" s="10" t="s">
+      <c r="L8" s="41" t="s">
         <v>33</v>
       </c>
-      <c r="L8" s="8" t="s">
+      <c r="M8" s="31"/>
+      <c r="N8" s="31"/>
+      <c r="P8" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="M8" s="10" t="s">
+      <c r="Q8" s="41" t="s">
         <v>35</v>
       </c>
+      <c r="R8" s="31" t="s">
+        <v>192</v>
+      </c>
+      <c r="S8" s="31"/>
     </row>
     <row r="9" spans="1:1025 16383:16384">
-      <c r="C9" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="D9" s="10"/>
+      <c r="C9" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="D9" s="25"/>
       <c r="F9" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="G9" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="I9" s="8" t="s">
+      <c r="H9" s="31"/>
+      <c r="I9" s="31"/>
+      <c r="K9" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="L9" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="L9" s="8" t="s">
+      <c r="M9" s="31"/>
+      <c r="N9" s="31"/>
+      <c r="P9" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="M9" s="10" t="s">
+      <c r="Q9" s="41" t="s">
         <v>43</v>
       </c>
+      <c r="R9" s="31" t="s">
+        <v>193</v>
+      </c>
+      <c r="S9" s="31"/>
     </row>
     <row r="10" spans="1:1025 16383:16384">
-      <c r="C10" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="D10" s="10"/>
+      <c r="C10" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="D10" s="25"/>
       <c r="F10" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="G10" s="13" t="s">
+      <c r="G10" s="29" t="s">
         <v>53</v>
       </c>
-      <c r="I10" s="8" t="s">
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
+      <c r="K10" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J10" s="10" t="s">
+      <c r="L10" s="41" t="s">
         <v>49</v>
       </c>
-      <c r="L10" s="8" t="s">
+      <c r="M10" s="31"/>
+      <c r="N10" s="31"/>
+      <c r="P10" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="M10" s="10" t="s">
+      <c r="Q10" s="41" t="s">
         <v>51</v>
       </c>
+      <c r="R10" s="31" t="s">
+        <v>190</v>
+      </c>
+      <c r="S10" s="31"/>
     </row>
     <row r="11" spans="1:1025 16383:16384">
-      <c r="C11" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="D11" s="10"/>
+      <c r="C11" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="D11" s="25"/>
       <c r="F11" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="G11" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="I11" s="8" t="s">
+      <c r="G11" s="29" t="s">
+        <v>181</v>
+      </c>
+      <c r="H11" s="31"/>
+      <c r="I11" s="31"/>
+      <c r="K11" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="J11" s="10" t="s">
+      <c r="L11" s="36" t="s">
         <v>93</v>
       </c>
-      <c r="L11" s="8" t="s">
+      <c r="M11" s="31">
+        <v>75</v>
+      </c>
+      <c r="N11" s="31"/>
+      <c r="P11" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="M11" s="10"/>
+      <c r="Q11" s="39" t="s">
+        <v>184</v>
+      </c>
+      <c r="R11" s="31"/>
+      <c r="S11" s="31"/>
     </row>
     <row r="12" spans="1:1025 16383:16384">
-      <c r="C12" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="D12" s="10"/>
+      <c r="C12" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="D12" s="25"/>
       <c r="F12" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="G12" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="I12" s="8" t="s">
+      <c r="G12" s="29" t="s">
+        <v>182</v>
+      </c>
+      <c r="H12" s="31"/>
+      <c r="I12" s="31"/>
+      <c r="K12" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="J12" s="10" t="s">
+      <c r="L12" s="36" t="s">
         <v>99</v>
       </c>
-      <c r="L12" s="8" t="s">
+      <c r="M12" s="31">
+        <v>74</v>
+      </c>
+      <c r="N12" s="31"/>
+      <c r="P12" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="M12" s="10"/>
+      <c r="Q12" s="8"/>
+      <c r="R12" s="31"/>
+      <c r="S12" s="31"/>
     </row>
     <row r="13" spans="1:1025 16383:16384">
-      <c r="C13" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="D13" s="15" t="s">
+      <c r="C13" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="D13" s="26"/>
+      <c r="F13" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="G13" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="H13" s="31"/>
+      <c r="I13" s="31"/>
+      <c r="K13" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="L13" s="38" t="s">
+        <v>57</v>
+      </c>
+      <c r="M13" s="31">
+        <v>36</v>
+      </c>
+      <c r="N13" s="31"/>
+      <c r="P13" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q13" s="41" t="s">
+        <v>71</v>
+      </c>
+      <c r="R13" s="35" t="s">
+        <v>194</v>
+      </c>
+      <c r="S13" s="31"/>
+    </row>
+    <row r="14" spans="1:1025 16383:16384">
+      <c r="C14" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="F13" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="I13" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="J13" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="L13" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="M13" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q13"/>
-    </row>
-    <row r="14" spans="1:1025 16383:16384">
-      <c r="C14" s="8" t="s">
+      <c r="D14" s="26"/>
+      <c r="F14" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="G14" s="28" t="s">
+        <v>73</v>
+      </c>
+      <c r="H14" s="31"/>
+      <c r="I14" s="31"/>
+      <c r="K14" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="L14" s="38" t="s">
+        <v>64</v>
+      </c>
+      <c r="M14" s="31">
+        <v>37</v>
+      </c>
+      <c r="N14" s="31"/>
+      <c r="P14" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q14" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="R14" s="34" t="s">
+        <v>187</v>
+      </c>
+      <c r="S14" s="31"/>
+    </row>
+    <row r="15" spans="1:1025 16383:16384">
+      <c r="C15" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="D14" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="I14" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="J14" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="L14" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="M14" s="30">
-        <v>46274</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1025 16383:16384">
-      <c r="C15" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="10"/>
+      <c r="F15" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="G15" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="H15" s="31"/>
+      <c r="I15" s="31"/>
+      <c r="K15" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="L15" s="38" t="s">
+        <v>69</v>
+      </c>
+      <c r="M15" s="31">
+        <v>38</v>
+      </c>
+      <c r="N15" s="31"/>
+      <c r="P15" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q15" s="39" t="s">
+        <v>83</v>
+      </c>
+      <c r="R15" s="31"/>
+      <c r="S15" s="31"/>
+    </row>
+    <row r="16" spans="1:1025 16383:16384">
+      <c r="C16" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="D16" s="39" t="s">
+        <v>116</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="G16" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="H16" s="31"/>
+      <c r="I16" s="31"/>
+      <c r="K16" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="L16" s="38" t="s">
+        <v>75</v>
+      </c>
+      <c r="M16" s="31">
+        <v>40</v>
+      </c>
+      <c r="N16" s="31"/>
+      <c r="P16" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="Q16" s="39" t="s">
+        <v>89</v>
+      </c>
+      <c r="R16" s="31"/>
+      <c r="S16" s="31"/>
+    </row>
+    <row r="17" spans="3:19">
+      <c r="C17" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="F15" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="I15" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="J15" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="L15" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="M15" s="10" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1025 16383:16384">
-      <c r="C16" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="D16" s="15" t="s">
+      <c r="D17" s="10"/>
+      <c r="F17" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="G17" s="28" t="s">
+        <v>91</v>
+      </c>
+      <c r="H17" s="31"/>
+      <c r="I17" s="31"/>
+      <c r="K17" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="L17" s="38" t="s">
+        <v>81</v>
+      </c>
+      <c r="M17" s="31">
+        <v>41</v>
+      </c>
+      <c r="N17" s="31"/>
+      <c r="P17" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q17" s="39" t="s">
+        <v>95</v>
+      </c>
+      <c r="R17" s="31"/>
+      <c r="S17" s="31"/>
+    </row>
+    <row r="18" spans="3:19">
+      <c r="C18" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="D18" s="10"/>
+      <c r="F18" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="G18" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="H18" s="31"/>
+      <c r="I18" s="31"/>
+      <c r="K18" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="L18" s="38" t="s">
+        <v>87</v>
+      </c>
+      <c r="M18" s="31">
+        <v>42</v>
+      </c>
+      <c r="N18" s="31"/>
+      <c r="P18" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="Q18" s="39" t="s">
+        <v>101</v>
+      </c>
+      <c r="R18" s="31"/>
+      <c r="S18" s="31"/>
+    </row>
+    <row r="19" spans="3:19">
+      <c r="C19" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="F16" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="I16" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="J16" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="L16" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="M16" s="10" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="17" spans="3:13">
-      <c r="C17" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="D17" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="G17" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="I17" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="J17" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="L17" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="M17" s="10" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="18" spans="3:13">
-      <c r="C18" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="D18" s="15" t="s">
-        <v>132</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="G18" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="I18" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="J18" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="L18" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="M18" s="10" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="19" spans="3:13">
-      <c r="C19" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="D19" s="15" t="s">
-        <v>135</v>
-      </c>
+      <c r="D19" s="10"/>
       <c r="F19" s="3"/>
       <c r="G19" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I19" s="8" t="s">
+      <c r="K19" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="J19" s="10" t="s">
+      <c r="L19" s="37" t="s">
         <v>103</v>
       </c>
-      <c r="L19" s="6" t="s">
+      <c r="M19" s="31">
+        <v>73</v>
+      </c>
+      <c r="N19" s="31"/>
+      <c r="P19" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="M19" s="10" t="s">
+      <c r="Q19" s="40" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="20" spans="3:13" ht="14.4">
-      <c r="C20" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="D20" s="15" t="s">
-        <v>138</v>
-      </c>
-      <c r="F20" s="8" t="s">
+      <c r="R19" s="31"/>
+      <c r="S19" s="31"/>
+    </row>
+    <row r="20" spans="3:19" ht="14.4">
+      <c r="C20" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="D20" s="10"/>
+      <c r="F20" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="G20" s="9" t="s">
+      <c r="G20" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="I20" s="8" t="s">
+      <c r="H20" s="31"/>
+      <c r="I20" s="31"/>
+      <c r="K20" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="J20" s="10" t="s">
+      <c r="L20" s="37" t="s">
         <v>107</v>
       </c>
-      <c r="L20" s="6" t="s">
+      <c r="M20" s="31">
+        <v>72</v>
+      </c>
+      <c r="N20" s="31"/>
+      <c r="P20" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="M20" s="10" t="s">
+      <c r="Q20" s="40" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="21" spans="3:13" ht="14.4">
-      <c r="F21" s="8" t="s">
+      <c r="R20" s="31"/>
+      <c r="S20" s="31"/>
+    </row>
+    <row r="21" spans="3:19" ht="14.4">
+      <c r="F21" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="G21" s="11" t="s">
+      <c r="G21" s="33" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="22" spans="3:13" ht="14.4">
-      <c r="F22" s="8" t="s">
+      <c r="H21" s="31"/>
+      <c r="I21" s="31"/>
+    </row>
+    <row r="22" spans="3:19" ht="14.4">
+      <c r="F22" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="G22" s="11" t="s">
+      <c r="G22" s="33" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="23" spans="3:13" ht="14.4">
-      <c r="F23" s="8" t="s">
+      <c r="H22" s="31"/>
+      <c r="I22" s="31"/>
+    </row>
+    <row r="23" spans="3:19" ht="14.4">
+      <c r="F23" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="G23" s="11" t="s">
+      <c r="G23" s="33" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="24" spans="3:13" ht="14.4">
-      <c r="F24" s="8" t="s">
+      <c r="H23" s="31"/>
+      <c r="I23" s="31"/>
+    </row>
+    <row r="24" spans="3:19" ht="14.4">
+      <c r="F24" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="G24" s="11" t="s">
+      <c r="G24" s="33" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="25" spans="3:13" ht="14.4">
-      <c r="F25" s="8" t="s">
+      <c r="H24" s="31"/>
+      <c r="I24" s="31"/>
+    </row>
+    <row r="25" spans="3:19" ht="14.4">
+      <c r="F25" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="G25" s="11" t="s">
+      <c r="G25" s="33" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="26" spans="3:13" ht="14.4">
-      <c r="F26" s="8" t="s">
+      <c r="H25" s="31"/>
+      <c r="I25" s="31"/>
+    </row>
+    <row r="26" spans="3:19" ht="14.4">
+      <c r="F26" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="G26" s="11" t="s">
+      <c r="G26" s="33" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="27" spans="3:13" ht="14.4">
-      <c r="F27" s="8" t="s">
+      <c r="H26" s="31"/>
+      <c r="I26" s="31"/>
+    </row>
+    <row r="27" spans="3:19" ht="14.4">
+      <c r="F27" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="G27" s="11" t="s">
+      <c r="G27" s="33" t="s">
         <v>62</v>
       </c>
+      <c r="H27" s="31"/>
+      <c r="I27" s="31"/>
+    </row>
+    <row r="31" spans="3:19">
+      <c r="J31"/>
+    </row>
+    <row r="37" spans="2:17">
+      <c r="B37"/>
+    </row>
+    <row r="44" spans="2:17">
+      <c r="Q44" s="45"/>
     </row>
   </sheetData>
   <pageMargins left="0" right="0" top="0.39370078740157505" bottom="0.39370078740157505" header="0" footer="0"/>
@@ -3012,501 +3281,501 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="10.69921875" customWidth="1"/>
-    <col min="2" max="2" width="24.296875" style="16" customWidth="1"/>
-    <col min="3" max="3" width="14" style="16" customWidth="1"/>
-    <col min="4" max="4" width="7.19921875" style="17" customWidth="1"/>
-    <col min="5" max="5" width="5.296875" style="17" customWidth="1"/>
-    <col min="6" max="6" width="16.8984375" style="18" customWidth="1"/>
-    <col min="7" max="7" width="17.296875" style="16" customWidth="1"/>
+    <col min="2" max="2" width="24.296875" style="11" customWidth="1"/>
+    <col min="3" max="3" width="14" style="11" customWidth="1"/>
+    <col min="4" max="4" width="7.19921875" style="12" customWidth="1"/>
+    <col min="5" max="5" width="5.296875" style="12" customWidth="1"/>
+    <col min="6" max="6" width="16.8984375" style="13" customWidth="1"/>
+    <col min="7" max="7" width="17.296875" style="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:7">
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="23" t="s">
+        <v>129</v>
+      </c>
+      <c r="C3" s="14"/>
+      <c r="D3" s="16" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7">
+      <c r="B4" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>165</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7">
+      <c r="B5" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="20"/>
+    </row>
+    <row r="6" spans="2:7">
+      <c r="B6" s="18" t="s">
+        <v>136</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="20" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7">
+      <c r="B7" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="E7" s="19">
+        <v>1</v>
+      </c>
+      <c r="F7" s="20">
+        <v>12.13</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7">
+      <c r="B10" s="23" t="s">
+        <v>140</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7">
+      <c r="B11" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="E11" s="16" t="s">
+        <v>165</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="G11" s="16" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7">
+      <c r="B12" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="18"/>
+    </row>
+    <row r="13" spans="2:7" ht="27.6">
+      <c r="B13" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="D13" s="19" t="s">
+        <v>169</v>
+      </c>
+      <c r="E13" s="19">
+        <v>1</v>
+      </c>
+      <c r="F13" s="20" t="s">
+        <v>170</v>
+      </c>
+      <c r="G13" s="18"/>
+    </row>
+    <row r="14" spans="2:7">
+      <c r="B14" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="D14" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="E14" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="F14" s="20" t="s">
+        <v>171</v>
+      </c>
+      <c r="G14" s="18"/>
+    </row>
+    <row r="15" spans="2:7">
+      <c r="B15" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="E15" s="19">
+        <v>1</v>
+      </c>
+      <c r="F15" s="20">
+        <v>14</v>
+      </c>
+      <c r="G15" s="18"/>
+    </row>
+    <row r="16" spans="2:7">
+      <c r="B16" s="18"/>
+      <c r="C16" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="18"/>
+    </row>
+    <row r="17" spans="2:7">
+      <c r="B17" s="18"/>
+      <c r="C17" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="18"/>
+    </row>
+    <row r="18" spans="2:7">
+      <c r="B18" s="18" t="s">
+        <v>180</v>
+      </c>
+      <c r="C18" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="E18" s="19">
+        <v>1</v>
+      </c>
+      <c r="F18" s="20">
+        <v>15</v>
+      </c>
+      <c r="G18" s="18"/>
+    </row>
+    <row r="19" spans="2:7">
+      <c r="B19" s="18"/>
+      <c r="C19" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="18"/>
+    </row>
+    <row r="20" spans="2:7">
+      <c r="B20" s="18"/>
+      <c r="C20" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="18"/>
+    </row>
+    <row r="22" spans="2:7">
+      <c r="B22" s="23" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7">
+      <c r="B23" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="20"/>
+      <c r="G23" s="18"/>
+    </row>
+    <row r="24" spans="2:7">
+      <c r="B24" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="18"/>
+    </row>
+    <row r="25" spans="2:7">
+      <c r="B25" s="18" t="s">
+        <v>155</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>156</v>
+      </c>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="18"/>
+    </row>
+    <row r="26" spans="2:7">
+      <c r="B26" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="18"/>
+    </row>
+    <row r="27" spans="2:7">
+      <c r="B27" s="18" t="s">
+        <v>159</v>
+      </c>
+      <c r="C27" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="18"/>
+    </row>
+    <row r="28" spans="2:7">
+      <c r="B28" s="18" t="s">
+        <v>160</v>
+      </c>
+      <c r="C28" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="18"/>
+    </row>
+    <row r="29" spans="2:7">
+      <c r="B29" s="18" t="s">
+        <v>161</v>
+      </c>
+      <c r="C29" s="18" t="s">
+        <v>162</v>
+      </c>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="20"/>
+      <c r="G29" s="18"/>
+    </row>
+    <row r="31" spans="2:7">
+      <c r="B31" s="23" t="s">
+        <v>130</v>
+      </c>
+      <c r="D31" s="16" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7">
+      <c r="B32" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="D32" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="E32" s="16" t="s">
+        <v>165</v>
+      </c>
+      <c r="F32" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="G32" s="16" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7">
+      <c r="B33" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="C33" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="20"/>
+      <c r="G33" s="18"/>
+    </row>
+    <row r="35" spans="2:7">
+      <c r="B35" s="23" t="s">
         <v>139</v>
       </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="21" t="s">
+      <c r="D35" s="16" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="36" spans="2:7">
+      <c r="B36" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="C36" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="D36" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="E36" s="16" t="s">
+        <v>165</v>
+      </c>
+      <c r="F36" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="G36" s="16" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="37" spans="2:7">
+      <c r="B37" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="C37" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="D37" s="19" t="s">
+        <v>169</v>
+      </c>
+      <c r="E37" s="19">
+        <v>1</v>
+      </c>
+      <c r="F37" s="20" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="4" spans="2:7">
-      <c r="B4" s="20" t="s">
-        <v>141</v>
-      </c>
-      <c r="C4" s="20" t="s">
-        <v>142</v>
-      </c>
-      <c r="D4" s="21" t="s">
+      <c r="G37" s="18" t="s">
         <v>174</v>
       </c>
-      <c r="E4" s="21" t="s">
+    </row>
+    <row r="38" spans="2:7">
+      <c r="B38" s="18"/>
+      <c r="C38" s="18"/>
+      <c r="D38" s="19" t="s">
+        <v>169</v>
+      </c>
+      <c r="E38" s="19">
+        <v>1</v>
+      </c>
+      <c r="F38" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="G38" s="18" t="s">
         <v>175</v>
       </c>
-      <c r="F4" s="22" t="s">
+    </row>
+    <row r="39" spans="2:7">
+      <c r="B39" s="18"/>
+      <c r="C39" s="18"/>
+      <c r="D39" s="19" t="s">
+        <v>169</v>
+      </c>
+      <c r="E39" s="19">
+        <v>1</v>
+      </c>
+      <c r="F39" s="20" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="5" spans="2:7">
-      <c r="B5" s="23" t="s">
-        <v>143</v>
-      </c>
-      <c r="C5" s="23" t="s">
+      <c r="G39" s="18" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="41" spans="2:7">
+      <c r="B41" s="23" t="s">
         <v>144</v>
       </c>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24"/>
-      <c r="F5" s="25"/>
-    </row>
-    <row r="6" spans="2:7">
-      <c r="B6" s="23" t="s">
-        <v>146</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>147</v>
-      </c>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="25" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="7" spans="2:7">
-      <c r="B7" s="23" t="s">
-        <v>188</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="D7" s="24" t="s">
-        <v>178</v>
-      </c>
-      <c r="E7" s="24">
-        <v>1</v>
-      </c>
-      <c r="F7" s="25">
-        <v>12.13</v>
-      </c>
-    </row>
-    <row r="10" spans="2:7">
-      <c r="B10" s="28" t="s">
+    </row>
+    <row r="42" spans="2:7">
+      <c r="B42" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="C42" s="15" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="43" spans="2:7">
+      <c r="B43" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="C43" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="D10" s="21" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="11" spans="2:7">
-      <c r="B11" s="20" t="s">
-        <v>141</v>
-      </c>
-      <c r="C11" s="20" t="s">
-        <v>142</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>174</v>
-      </c>
-      <c r="E11" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="F11" s="22" t="s">
-        <v>176</v>
-      </c>
-      <c r="G11" s="21" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="12" spans="2:7">
-      <c r="B12" s="23" t="s">
-        <v>152</v>
-      </c>
-      <c r="C12" s="23" t="s">
+    </row>
+    <row r="45" spans="2:7">
+      <c r="B45" s="23" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="46" spans="2:7">
+      <c r="B46" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="C46" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="D46" s="19"/>
+      <c r="E46" s="19"/>
+      <c r="F46" s="20"/>
+      <c r="G46" s="18"/>
+    </row>
+    <row r="47" spans="2:7">
+      <c r="B47" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="D12" s="24"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="23"/>
-    </row>
-    <row r="13" spans="2:7" ht="27.6">
-      <c r="B13" s="23" t="s">
-        <v>155</v>
-      </c>
-      <c r="C13" s="23" t="s">
-        <v>156</v>
-      </c>
-      <c r="D13" s="24" t="s">
-        <v>179</v>
-      </c>
-      <c r="E13" s="24">
-        <v>1</v>
-      </c>
-      <c r="F13" s="25" t="s">
-        <v>180</v>
-      </c>
-      <c r="G13" s="23"/>
-    </row>
-    <row r="14" spans="2:7">
-      <c r="B14" s="23" t="s">
-        <v>157</v>
-      </c>
-      <c r="C14" s="23" t="s">
-        <v>158</v>
-      </c>
-      <c r="D14" s="24" t="s">
-        <v>181</v>
-      </c>
-      <c r="E14" s="24" t="s">
-        <v>181</v>
-      </c>
-      <c r="F14" s="25" t="s">
-        <v>181</v>
-      </c>
-      <c r="G14" s="23"/>
-    </row>
-    <row r="15" spans="2:7">
-      <c r="B15" s="23" t="s">
-        <v>189</v>
-      </c>
-      <c r="C15" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="D15" s="24" t="s">
-        <v>178</v>
-      </c>
-      <c r="E15" s="24">
-        <v>1</v>
-      </c>
-      <c r="F15" s="25">
-        <v>14</v>
-      </c>
-      <c r="G15" s="23"/>
-    </row>
-    <row r="16" spans="2:7">
-      <c r="B16" s="23"/>
-      <c r="C16" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="23"/>
-    </row>
-    <row r="17" spans="2:7">
-      <c r="B17" s="23"/>
-      <c r="C17" s="27" t="s">
-        <v>37</v>
-      </c>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="23"/>
-    </row>
-    <row r="18" spans="2:7">
-      <c r="B18" s="23" t="s">
-        <v>190</v>
-      </c>
-      <c r="C18" s="27" t="s">
-        <v>45</v>
-      </c>
-      <c r="D18" s="24" t="s">
-        <v>178</v>
-      </c>
-      <c r="E18" s="24">
-        <v>1</v>
-      </c>
-      <c r="F18" s="25">
-        <v>15</v>
-      </c>
-      <c r="G18" s="23"/>
-    </row>
-    <row r="19" spans="2:7">
-      <c r="B19" s="23"/>
-      <c r="C19" s="27" t="s">
-        <v>53</v>
-      </c>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="23"/>
-    </row>
-    <row r="20" spans="2:7">
-      <c r="B20" s="23"/>
-      <c r="C20" s="29" t="s">
-        <v>60</v>
-      </c>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="23"/>
-    </row>
-    <row r="22" spans="2:7">
-      <c r="B22" s="28" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="23" spans="2:7">
-      <c r="B23" s="20" t="s">
-        <v>141</v>
-      </c>
-      <c r="C23" s="20" t="s">
-        <v>142</v>
-      </c>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="23"/>
-    </row>
-    <row r="24" spans="2:7">
-      <c r="B24" s="23" t="s">
-        <v>164</v>
-      </c>
-      <c r="C24" s="23" t="s">
-        <v>77</v>
-      </c>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="23"/>
-    </row>
-    <row r="25" spans="2:7">
-      <c r="B25" s="23" t="s">
-        <v>165</v>
-      </c>
-      <c r="C25" s="23" t="s">
-        <v>166</v>
-      </c>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="23"/>
-    </row>
-    <row r="26" spans="2:7">
-      <c r="B26" s="23" t="s">
-        <v>167</v>
-      </c>
-      <c r="C26" s="23" t="s">
-        <v>168</v>
-      </c>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="23"/>
-    </row>
-    <row r="27" spans="2:7">
-      <c r="B27" s="23" t="s">
-        <v>169</v>
-      </c>
-      <c r="C27" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="25"/>
-      <c r="G27" s="23"/>
-    </row>
-    <row r="28" spans="2:7">
-      <c r="B28" s="23" t="s">
-        <v>170</v>
-      </c>
-      <c r="C28" s="23" t="s">
-        <v>124</v>
-      </c>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="23"/>
-    </row>
-    <row r="29" spans="2:7">
-      <c r="B29" s="23" t="s">
-        <v>171</v>
-      </c>
-      <c r="C29" s="23" t="s">
-        <v>172</v>
-      </c>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="25"/>
-      <c r="G29" s="23"/>
-    </row>
-    <row r="31" spans="2:7">
-      <c r="B31" s="28" t="s">
-        <v>140</v>
-      </c>
-      <c r="D31" s="21" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="32" spans="2:7">
-      <c r="B32" s="20" t="s">
-        <v>141</v>
-      </c>
-      <c r="C32" s="20" t="s">
-        <v>142</v>
-      </c>
-      <c r="D32" s="21" t="s">
-        <v>174</v>
-      </c>
-      <c r="E32" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="F32" s="22" t="s">
-        <v>176</v>
-      </c>
-      <c r="G32" s="21" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="33" spans="2:7">
-      <c r="B33" s="23" t="s">
-        <v>145</v>
-      </c>
-      <c r="C33" s="23" t="s">
-        <v>145</v>
-      </c>
-      <c r="D33" s="24"/>
-      <c r="E33" s="24"/>
-      <c r="F33" s="25"/>
-      <c r="G33" s="23"/>
-    </row>
-    <row r="35" spans="2:7">
-      <c r="B35" s="28" t="s">
-        <v>149</v>
-      </c>
-      <c r="D35" s="21" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="36" spans="2:7">
-      <c r="B36" s="20" t="s">
-        <v>141</v>
-      </c>
-      <c r="C36" s="20" t="s">
-        <v>142</v>
-      </c>
-      <c r="D36" s="21" t="s">
-        <v>174</v>
-      </c>
-      <c r="E36" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="F36" s="22" t="s">
-        <v>176</v>
-      </c>
-      <c r="G36" s="21" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="37" spans="2:7">
-      <c r="B37" s="23" t="s">
-        <v>151</v>
-      </c>
-      <c r="C37" s="23" t="s">
-        <v>25</v>
-      </c>
-      <c r="D37" s="24" t="s">
-        <v>179</v>
-      </c>
-      <c r="E37" s="24">
-        <v>1</v>
-      </c>
-      <c r="F37" s="25" t="s">
-        <v>183</v>
-      </c>
-      <c r="G37" s="23" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="38" spans="2:7">
-      <c r="B38" s="23"/>
-      <c r="C38" s="23"/>
-      <c r="D38" s="24" t="s">
-        <v>179</v>
-      </c>
-      <c r="E38" s="24">
-        <v>1</v>
-      </c>
-      <c r="F38" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="G38" s="23" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="39" spans="2:7">
-      <c r="B39" s="23"/>
-      <c r="C39" s="23"/>
-      <c r="D39" s="24" t="s">
-        <v>179</v>
-      </c>
-      <c r="E39" s="24">
-        <v>1</v>
-      </c>
-      <c r="F39" s="25" t="s">
-        <v>186</v>
-      </c>
-      <c r="G39" s="23" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="41" spans="2:7">
-      <c r="B41" s="28" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="42" spans="2:7">
-      <c r="B42" s="20" t="s">
-        <v>141</v>
-      </c>
-      <c r="C42" s="20" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="43" spans="2:7">
-      <c r="B43" s="23" t="s">
-        <v>159</v>
-      </c>
-      <c r="C43" s="23" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="45" spans="2:7">
-      <c r="B45" s="28" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="46" spans="2:7">
-      <c r="B46" s="20" t="s">
-        <v>141</v>
-      </c>
-      <c r="C46" s="20" t="s">
-        <v>142</v>
-      </c>
-      <c r="D46" s="24"/>
-      <c r="E46" s="24"/>
-      <c r="F46" s="25"/>
-      <c r="G46" s="23"/>
-    </row>
-    <row r="47" spans="2:7">
-      <c r="B47" s="23" t="s">
-        <v>163</v>
-      </c>
-      <c r="C47" s="23" t="s">
+      <c r="C47" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D47" s="24"/>
-      <c r="E47" s="24"/>
-      <c r="F47" s="25"/>
-      <c r="G47" s="23"/>
+      <c r="D47" s="19"/>
+      <c r="E47" s="19"/>
+      <c r="F47" s="20"/>
+      <c r="G47" s="18"/>
     </row>
     <row r="48" spans="2:7">
-      <c r="B48" s="23"/>
-      <c r="C48" s="23" t="s">
+      <c r="B48" s="18"/>
+      <c r="C48" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="D48" s="24"/>
-      <c r="E48" s="24"/>
-      <c r="F48" s="25"/>
-      <c r="G48" s="23"/>
+      <c r="D48" s="19"/>
+      <c r="E48" s="19"/>
+      <c r="F48" s="20"/>
+      <c r="G48" s="18"/>
     </row>
   </sheetData>
   <pageMargins left="0" right="0" top="0.39370078740157505" bottom="0.39370078740157505" header="0" footer="0"/>

</xml_diff>